<commit_message>
Otomatik veri güncelleme (10.09.2026 15:11 UTC)
</commit_message>
<xml_diff>
--- a/hazine nakit/nakit.xlsx
+++ b/hazine nakit/nakit.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N235"/>
+  <dimension ref="A1:N236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10683,7 +10683,7 @@
         <v>7</v>
       </c>
       <c r="D235" t="n">
-        <v>1394899.46</v>
+        <v>1394242.24</v>
       </c>
       <c r="E235" t="n">
         <v>1790549.48</v>
@@ -10695,16 +10695,16 @@
         <v>325909.94</v>
       </c>
       <c r="H235" t="n">
-        <v>-69740.08</v>
+        <v>-70397.3</v>
       </c>
       <c r="I235" t="n">
-        <v>0</v>
+        <v>609.34</v>
       </c>
       <c r="J235" t="n">
-        <v>-395650.02</v>
+        <v>-395697.9</v>
       </c>
       <c r="K235" t="n">
-        <v>395650.02</v>
+        <v>395697.9</v>
       </c>
       <c r="L235" t="n">
         <v>315730.84</v>
@@ -10714,6 +10714,50 @@
       </c>
       <c r="N235" t="n">
         <v>116485.82</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B236" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C236" t="n">
+        <v>8</v>
+      </c>
+      <c r="D236" t="n">
+        <v>1677103.89</v>
+      </c>
+      <c r="E236" t="n">
+        <v>1627287.79</v>
+      </c>
+      <c r="F236" t="n">
+        <v>1467506.52</v>
+      </c>
+      <c r="G236" t="n">
+        <v>159781.27</v>
+      </c>
+      <c r="H236" t="n">
+        <v>209597.37</v>
+      </c>
+      <c r="I236" t="n">
+        <v>0</v>
+      </c>
+      <c r="J236" t="n">
+        <v>49816.1</v>
+      </c>
+      <c r="K236" t="n">
+        <v>-49816.1</v>
+      </c>
+      <c r="L236" t="n">
+        <v>149418.44</v>
+      </c>
+      <c r="M236" t="n">
+        <v>166432.97</v>
+      </c>
+      <c r="N236" t="n">
+        <v>-17014.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>